<commit_message>
💡 Updated logic.py to fix amount parsing and improve Excel formatting
</commit_message>
<xml_diff>
--- a/data/voice_expenses.xlsx
+++ b/data/voice_expenses.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Expense Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -16,10 +16,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-  </numFmts>
-  <fonts count="3">
+  <numFmts count="0"/>
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -30,33 +28,16 @@
     <font>
       <b val="1"/>
     </font>
-    <font>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="12"/>
-    </font>
   </fonts>
-  <fills count="4">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="001F4E78"/>
-        <bgColor rgb="001F4E78"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F2F2F2"/>
-        <bgColor rgb="00F2F2F2"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="3">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -70,43 +51,14 @@
       <top style="thin"/>
       <bottom style="thin"/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="00CCCCCC"/>
-      </left>
-      <right style="thin">
-        <color rgb="00CCCCCC"/>
-      </right>
-      <top style="thin">
-        <color rgb="00CCCCCC"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00CCCCCC"/>
-      </bottom>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -182,145 +134,6 @@
     </indexedColors>
   </colors>
 </styleSheet>
-</file>
-
-<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <chart>
-    <title>
-      <tx>
-        <rich>
-          <a:bodyPr/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr/>
-            </a:pPr>
-            <a:r>
-              <a:t>Spending by Category</a:t>
-            </a:r>
-          </a:p>
-        </rich>
-      </tx>
-    </title>
-    <plotArea>
-      <barChart>
-        <barDir val="col"/>
-        <grouping val="clustered"/>
-        <ser>
-          <idx val="0"/>
-          <order val="0"/>
-          <tx>
-            <strRef>
-              <f>'Expense Summary'!C1</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <numRef>
-              <f>'Expense Summary'!$B$2:$B$5</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Expense Summary'!$C$2:$C$5</f>
-            </numRef>
-          </val>
-        </ser>
-        <gapWidth val="150"/>
-        <axId val="10"/>
-        <axId val="100"/>
-      </barChart>
-      <catAx>
-        <axId val="10"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <axPos val="l"/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>Category</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="100"/>
-        <lblOffset val="100"/>
-      </catAx>
-      <valAx>
-        <axId val="100"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <axPos val="l"/>
-        <majorGridlines/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>Amount ($)</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="10"/>
-      </valAx>
-    </plotArea>
-    <legend>
-      <legendPos val="r"/>
-    </legend>
-    <plotVisOnly val="1"/>
-    <dispBlanksAs val="gap"/>
-  </chart>
-</chartSpace>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <oneCellAnchor>
-    <from>
-      <col>0</col>
-      <colOff>0</colOff>
-      <row>8</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="5400000" cy="2700000"/>
-    <graphicFrame>
-      <nvGraphicFramePr>
-        <cNvPr id="1" name="Chart 1"/>
-        <cNvGraphicFramePr/>
-      </nvGraphicFramePr>
-      <xfrm/>
-      <a:graphic>
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
-        </a:graphicData>
-      </a:graphic>
-    </graphicFrame>
-    <clientData/>
-  </oneCellAnchor>
-</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -612,131 +425,32 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="57" customWidth="1" min="4" max="4"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Date/Time</t>
+          <t>Date</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Amount ($)</t>
+          <t>Amount</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="3" t="inlineStr">
-        <is>
-          <t>2025-10-13</t>
-        </is>
-      </c>
-      <c r="B2" s="3" t="inlineStr">
-        <is>
-          <t>Food</t>
-        </is>
-      </c>
-      <c r="C2" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="D2" s="3" t="inlineStr">
-        <is>
-          <t>Today I spent ten dollars on gas.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="5" t="inlineStr">
-        <is>
-          <t>2025-10-13</t>
-        </is>
-      </c>
-      <c r="B3" s="5" t="inlineStr">
-        <is>
-          <t>Transportation</t>
-        </is>
-      </c>
-      <c r="C3" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="D3" s="5" t="inlineStr">
-        <is>
-          <t>Two days ago, I spent five dollars on a train ticket.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>2025-10-12</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>Food</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>Yesterday I spent seven dollars on a train ticket.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="5" t="inlineStr">
-        <is>
-          <t>2025-10-13</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="inlineStr">
-        <is>
-          <t>Food</t>
-        </is>
-      </c>
-      <c r="C5" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="D5" s="5" t="inlineStr">
-        <is>
-          <t>Today I spent five dollars on a train ticket.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="3" t="inlineStr"/>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="n">
-        <v>29</v>
-      </c>
-      <c r="D6" s="3" t="inlineStr"/>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Finalize SpendLens v1.0 — 100% tests passed, SOLID + TDD implemented
</commit_message>
<xml_diff>
--- a/data/voice_expenses.xlsx
+++ b/data/voice_expenses.xlsx
@@ -425,13 +425,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Date</t>
+          <t>Date/Time</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
@@ -441,12 +441,32 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Amount</t>
+          <t>Amount ($)</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2025-10-27</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Shopping</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>I went to the shop and bought three dollars worth of shoes.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: remove TOTAL row from Excel export chart generation
</commit_message>
<xml_diff>
--- a/data/voice_expenses.xlsx
+++ b/data/voice_expenses.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -450,26 +450,6 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>2025-10-27</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Shopping</t>
-        </is>
-      </c>
-      <c r="C2" t="n">
-        <v>3</v>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>I went to the shop and bought three dollars worth of shoes.</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>